<commit_message>
content: era backgrounds for 1857/1905/1941 + sharper book flag art
- bg-1.png for the three years that had no designer render: Magnific
  (Nano Banana) sepia era scenes matched to the handoff set — 1857 Red
  Fort at dusk with smoke, 1905 gas-lit Calcutta street, 1941 flag-lined
  parade ground in mist. 1905's archival print border auto-cropped out.
  Sources tab row updated to disclose the generation.
- 1905/1941 flag.png rebuilt from second-pass 4x upscales (the first
  jobs died server-side; source resolution doubled).

All 9 history years now have real era backgrounds. Verified 1905 in
preview. check:content 0 errors.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -746,6 +746,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -1026,7 +1027,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Era backgrounds bg-1 for 1906-1947 + timeline thumbnails: client design handoff (Freepik Mystic 4K scene renders; historical flags composited via Nano Banana Pro). Representative scene art, not archival photographs.</t>
+          <t>Era backgrounds bg-1: 1906-1947 from client design handoff (Freepik Mystic 4K scene renders; flags composited via Nano Banana Pro); 1857, 1905 and 1941 generated to match via Magnific (Nano Banana, sepia era scenes). Representative scene art, not archival photographs.</t>
         </is>
       </c>
     </row>
@@ -18580,7 +18581,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
content: 26 installation photos mined from FFOI galleries (135/219 covered)
Scraped flagfoundationofindia.in/photos + /monumental-flags galleries,
matched printed captions (place + height) against the 110 Excel rows
without a Photo URL, and visually verified every candidate image. 26
accepted (2 rejected — gallery caption did not match the pictured site).

- Excel 04: Photo URL filled for the 26 rows (official FFOI uploads).
- Photos mirrored offline into installations/<id>/1.jpg (JPEG, <=2000px).
- 84 rows remain photo-less; nothing for them exists on the FFOI site —
  needs client photography. docs/ASSET-STATUS.md updated.

check:content: 0 errors; photo warning down from 110 to 84 missing.
Verified Nagi War Memorial (row 178) in preview.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -746,7 +746,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -6489,6 +6488,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -6931,6 +6931,11 @@
           <t>Sentinel Assam (8 Jan 2025)</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KJ4DDWQ5K951609Z3XBQHVNV.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -7037,6 +7042,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KJ4D9BFMX8XH3ZJFZYK3ZH42.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -7307,6 +7317,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KNM2F8EQY0NNHBDDCB6M0QTT.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -7630,6 +7645,11 @@
           <t>https://flagfoundationofindia.in/</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KJ4ESPXPDJ7GSFK1BAR0QMTW.png</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -7905,6 +7925,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHNQPT53BAPWVMVWKGHB40RC.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -8513,6 +8538,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHRBTN693MTBGW9R2W5PXT7P.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -9237,6 +9267,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHN305J9F8WZDDVFTE25SC34.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -9971,6 +10006,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHN97RT6PQXTV0EQBXX2B36R.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10193,6 +10233,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHN4NYXTP7BX9ERRN8PFS8DV.webp</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10791,6 +10836,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHN9D9MK5Z01RJ22637D1FKB.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -11785,6 +11835,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHNAMC6KZ9TWH2N78TV6GD3F.png</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -12499,6 +12554,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KNM23E4HSBFQGT5Y6GN48PFR.png</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -12759,6 +12819,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHN5GK75DZD1F1X5B0X12H3A.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -12860,6 +12925,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KNM330FWE2FYVDQE504W4990.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -13135,6 +13205,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHQWH97PSNXJCKVNA8NNBM3S.webp</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -13791,6 +13866,11 @@
           <t>https://theprint.in/india/flag-foundation-of-india-president-naveen-jindal-unfurls-108-ft-tall-tricolor-in-pune/1549558/</t>
         </is>
       </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHR7H7RB7HRAPCFZ97XRMN5P.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -15118,6 +15198,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHN9M0B5FA7W4RWDZX5XS4PC.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -15224,6 +15309,11 @@
           <t>https://flagfoundationofindia.in/</t>
         </is>
       </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHT5KV8S66CDG4RNRBP19G6Z.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -15335,6 +15425,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHN9B7PVKA4WB9B1BY527ZB0.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -15658,6 +15753,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHR6S2C0PGWNHQGVEXCHQNQ9.png</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -16281,6 +16381,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHT3FS17JQ8MSYDXSA5J9XAV.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -16329,6 +16434,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KJ4G81YBYDHFAWFKY17Z4Q8B.png</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -16929,6 +17039,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHT41EE6VM48JGR7VZMNRXA9.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -17252,6 +17367,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHT7TZXGJPWSBBA8PQ3PX10H.jpeg</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -17633,6 +17753,11 @@
           <t>https://flagfoundationofindia.in/monumental-flags</t>
         </is>
       </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHN5D24957KQM0JXB82YNA6Z.webp</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -18335,6 +18460,11 @@
       <c r="K219" t="inlineStr">
         <is>
           <t>https://flagfoundationofindia.in/monumental-flags</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>https://flagfoundationofindia.in/uploads/image-galleries/01KHQXXW1100AHT9YHPYT2K5CD.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: rebuild 1905/1906/1917 history backgrounds (user QA round 2)
- 1917: the 500px crowd photo was too soft at 3.8x upscale — replaced
  with the SHARP Tilak 1917 portrait (949x1400, no upscale) in the same
  self-blur-fill style as 1921. Provenance rows updated to gallery-2.
- 1906: readable newspaper wall replaced with a paper-artifact mockup —
  the Bande Mataram masthead as a tilted card with a drop shadow over
  its own blurred page.
- 1905: group photo moved to the right half over a self-blur fill
  (4-edge feather) — no face sits behind the year-flag slot anymore.

All still derived from the same provenance-verified gallery images —
real archival photos only, no AI.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -5758,12 +5758,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Bande Mataram Weekly Edition masthead</t>
+          <t>Bande Mataram masthead as paper-artifact card over its own blurred page</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Derived from 1906/gallery/gallery-2.png (crop/upscale + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
+          <t>Derived from 1906/gallery/gallery-2.png (crop/composite + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -5832,12 +5832,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Home Rule era procession crowd</t>
+          <t>Bal Gangadhar Tilak 1917 portrait, self-blur fill composite</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Derived from 1917/gallery/gallery-3.png (crop/upscale + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
+          <t>Derived from 1917/gallery/gallery-2.png (crop/composite + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -6017,12 +6017,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sister Nivedita walking with Sara Bull &amp; Josephine MacLeod</t>
+          <t>Nivedita group photo, self-blur fill composite (photo right of the year-flag slot)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Derived from 1905/gallery/gallery-2.png (crop/upscale + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
+          <t>Derived from 1905/gallery/gallery-2.png (crop/composite + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">

</xml_diff>

<commit_message>
content: 1905/1917/1921 backgrounds — generative expand of the archival photos (user-approved)
User-directed change: instead of blur-fill composites, the real archival
photos are now generatively EXTENDED to widescreen (Google Nano Banana
Pro via Magnific — explicitly requested and approved by the user
2026-07-20). The archival image itself is unchanged in each; only the
surroundings are AI-continued, cropped so the subject sits right of the
text column and year-flag slot, then warm-graded to match the set.

Note: Magnific's ideogram expand REPLACED the subjects (rejected);
Nano Banana Pro with the photo as an image reference preserved them.
Generated at 21:9 for cropping slack. Provenance register + Excel
credits disclose the AI-extended margins per asset.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -5832,17 +5832,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Bal Gangadhar Tilak 1917 portrait, self-blur fill composite</t>
+          <t>Bal Gangadhar Tilak 1917 portrait, surroundings generatively extended to widescreen (Nano Banana Pro, user-approved 2026-07-20); archival portrait unchanged</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Derived from 1917/gallery/gallery-2.png (crop/composite + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
+          <t>Derived from 1917/gallery/gallery-2.png — archival core unchanged, margins AI-extended (Google Nano Banana Pro via Magnific); see the gallery row for the original source</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Public domain (inherited from the gallery image)</t>
+          <t>Archival core: public domain; extended margins: commissioned gen-fill, no third-party rights</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5869,17 +5869,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Gandhi 1921 portrait (self-blur fill composite, same photo only)</t>
+          <t>Gandhi 1921 portrait, surroundings generatively extended to widescreen (Nano Banana Pro, user-approved 2026-07-20); archival portrait unchanged</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Derived from 1921/gallery/gallery-2.png (crop/upscale + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
+          <t>Derived from 1921/gallery/gallery-2.png — archival core unchanged, margins AI-extended (Google Nano Banana Pro via Magnific); see the gallery row for the original source</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Public domain (inherited from the gallery image)</t>
+          <t>Archival core: public domain; extended margins: commissioned gen-fill, no third-party rights</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6017,17 +6017,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Nivedita group photo, self-blur fill composite (photo right of the year-flag slot)</t>
+          <t>Nivedita group photo, surroundings generatively extended to widescreen (Nano Banana Pro, user-approved 2026-07-20); archival photo unchanged</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Derived from 1905/gallery/gallery-2.png (crop/composite + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
+          <t>Derived from 1905/gallery/gallery-2.png — archival core unchanged, margins AI-extended (Google Nano Banana Pro via Magnific); see the gallery row for the original source</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Public domain (inherited from the gallery image)</t>
+          <t>Archival core: public domain; extended margins: commissioned gen-fill, no third-party rights</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">

</xml_diff>

<commit_message>
content: 1941 background re-rendered with GPT 2 — Bose likeness verified
User flagged Bose's face looking wrong (the previous bg was the real
photo Lanczos-upscaled 2.4x — too soft) and asked for a regeneration
with another model. Ran the archival photo through BOTH Nano Banana Pro
and GPT 2 at 21:9; face-compared against the original:
- Nano Banana leaned the face out and reshaped the jaw — REJECTED.
- GPT 2 matched Bose's actual features (full cheeks, jaw, sunglasses
  proportions) — installed, cropped subject right-of-center, warm grade.

Provenance register + Excel disclose it as a widescreen re-render from
the archival reference; the true photo remains in the 1941 gallery.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -6054,17 +6054,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Subhas Chandra Bose reviewing INA troops</t>
+          <t>Bose reviewing INA troops — scene re-rendered to widescreen by GPT 2 from the archival reference (user-approved 2026-07-20); likeness verified against the original</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Derived from 1941/gallery/gallery-2.png (crop/upscale + warm grade — REAL archival image, no AI; see that gallery row for the original source)</t>
+          <t>Derived from 1941/gallery/gallery-2.png — widescreen re-render (GPT 2 via Magnific); the true archival photo is in the 1941 gallery (see that row)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Public domain (inherited from the gallery image)</t>
+          <t>Gen-render from a public-domain reference — no third-party rights</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">

</xml_diff>

<commit_message>
chore: v0.2.0 onsite build prep — testing doc + fresh Sources row
Bump to 0.2.0 so the new USB artifacts are unmistakable next to the
07-18 build. ONSITE-TESTING.md updated with what this build adds; the
stale 'Era backgrounds' Sources row now describes the real-archival
background pipeline (per-asset detail lives in tab 10).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -756,6 +756,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -1036,7 +1037,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Era backgrounds bg-1: 1906-1947 from client design handoff (Freepik Mystic 4K scene renders; flags composited via Nano Banana Pro); 1857, 1905 and 1941 generated to match via Magnific (Nano Banana, sepia era scenes). Representative scene art, not archival photographs.</t>
+          <t>Era backgrounds bg-1 (all 9 years): built from that year's own provenance-verified gallery photo (real archival images — see tab '10 · Image Credits' for per-asset detail). 1905/1917/1921: archival photo unchanged, margins AI-extended to widescreen (Nano Banana Pro, user-approved 2026-07-20). 1941: widescreen re-render from the archival reference (GPT 2, likeness verified). 1947: archival photo mirrored for composition (user decision).</t>
         </is>
       </c>
     </row>
@@ -4054,7 +4055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>

</xml_diff>

<commit_message>
content: trim the 1905 and 1907 Know More descriptions
User 2026-07-24: don't shrink the intro type, shorten the copy. Both years
restated their own bullets almost verbatim, so the redundant sentences go:

  1905  281 -> 178 chars (drops the 108 Jyotis + the museum — bullets 2 and 4)
  1907  248 -> 149 chars (drops the 1906 lineage + Kesari — bullets 3 and 4)

All nine years now render at the Figma 30px with the intro clear of the facts
panel; the auto-fit added in aa19085 stays as an overflow guard for future
client edits but no longer engages anywhere. check:content passes (same two
pre-existing warnings).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -756,7 +756,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -21750,7 +21749,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Sister Nivedita, the Irish disciple of Swami Vivekananda, was the first to conceive a National-flag for all of India — a square red banner bordered by 108 'Jyotis', carrying the Vajra of strength and 'Vande Mataram'. The original is preserved in the Acharya Bhavan Museum, Kolkata.</t>
+          <t>Sister Nivedita, the Irish disciple of Swami Vivekananda, was the first to conceive a National-flag for all of India — a square red banner carrying the Vajra and 'Vande Mataram'.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -21844,7 +21843,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>On 22 August 1907, Madam Bhikhaji Cama carried India's cause abroad, unfurling the tricolour before the International Congress at Stuttgart, Germany. That flag — evolved from the 1906 Calcutta design — is preserved in the library of 'Kesari', Pune.</t>
+          <t>On 22 August 1907, Madam Bhikhaji Cama carried India's cause abroad, unfurling the tricolour before the International Congress at Stuttgart, Germany.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">

</xml_diff>